<commit_message>
Document the Fixed Effects role in Regression Instructions
Adds the panel Fixed Effects role to the Role bullet list so users know
it absorbs a per-group intercept (one-way within transformation) and
that Type/Reference Level don't apply to that row. Regenerated the
static template so the shipped sheet matches.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/static_sheets.xlsx
+++ b/templates/static_sheets.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Stephen_Colodner\windows code\Statistical_Analysis_Lambda_Catalog\.claude\worktrees\residual-headers-conditionals-021ab5\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Stephen_Colodner\windows code\Statistical_Analysis_Lambda_Catalog\.claude\worktrees\bridge-cse_01CECbFAThBCAdeR5ZRcns7Y\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9F65382-2CF4-4770-9945-DD862A38544B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A4277C5C-F7C6-406E-A4F7-783169E2384B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2895" yWindow="1050" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{1411C739-6A2D-448E-B19F-D2DD9A0E5CC5}"/>
+    <workbookView xWindow="3120" yWindow="3120" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{1411C739-6A2D-448E-B19F-D2DD9A0E5CC5}"/>
   </bookViews>
   <sheets>
     <sheet name="Regression Instructions" sheetId="2" r:id="rId1"/>
@@ -60,322 +60,323 @@
     <t>Define your model in the MODEL SPECIFICATION block (columns A–L):</t>
   </si>
   <si>
+    <t>For each included Predictor, set its Type. Continuous predictors enter the design matrix as-is. Categorical predictors are dummy-coded automatically: each level except the reference level becomes a 0/1 column with a level-qualified name (e.g. "Status: Developing"). The reference level defaults to the first level in sort order; type a level into Reference Level to override it (the cell turns red if that level does not exist in the analysis sample). The Levels and Reference In Use columns display what the model will do: the distinct level count in the analysis sample, and the reference actually in effect. A categorical with one level (or an invalid reference) is flagged red and contributes no columns — the rest of the model still computes.</t>
+  </si>
+  <si>
+    <t>If your table has more columns than the shipped dataset, fill in Role, Include, and Type for the extra specification rows — the dropdowns are available all the way down. A row with a blank Role is ignored. The Order and Transform columns are placeholders for a future version and are not read by any formula; they are hidden on the sheet. The Sequence column marks at most one variable as the ordering axis for future lag/difference/serial-correlation features — it is independent of Role and Type (a Predictor can also be the sequence axis). Leave it blank for non-panel data; marking two or more rows shows a red error in the status cell above the column. The Sequence Period column (I) is the typed override input: type a number on the flagged row to declare a Δ that differs from the candidate. The Period In Use column (J) is the live companion — it shows the typed override if column I is non-blank, otherwise the computed candidate (the most common gap between consecutive periods within a group). Lag_By and Difference_By fall back to Base_Period_Delta() when their [delta] argument is omitted — never a silent 1.</t>
+  </si>
+  <si>
+    <t>Intercept:</t>
+  </si>
+  <si>
+    <t>The Intercept toggle sits at the top of the Include column (C2). Leave it TRUE for models with Categorical predictors: reference-level dummy coding relies on the intercept to carry the baseline, and the toggle flags red if it is FALSE while a Categorical predictor is included.</t>
+  </si>
+  <si>
+    <t>Which rows are used:</t>
+  </si>
+  <si>
+    <t>The analysis sample is derived automatically — a row is included when the Response is numeric, every included Continuous predictor is numeric, and every Filter column is truthy. There is nothing to configure beyond the Roles. Note that Categorical predictors impose no completeness requirement: rows with a blank category still enter the sample (all of that variable's dummies are blank there) unless a Filter excludes them.</t>
+  </si>
+  <si>
+    <t>Optional — point prediction:</t>
+  </si>
+  <si>
+    <t>Enter a value for each design-matrix column in the orange cells under PREDICTION INPUTS (column AH) — one row per constructed column, including one per dummy (use 1 for the scenario's level, 0 for its siblings; no Intercept row — the model's own baseline is handled automatically). The Training Mean column beside the inputs shows each column's mean over the analysis sample, which is also the prefilled default — so the untouched prediction is at the data's center. Results appear in the PREDICTION OUTPUTS box above as both a mean-response confidence interval (CI) and a wider new-observation prediction interval (PI); the confidence level is controlled by the Alpha cell (Y12) in REGRESSION OUTPUTS. If a Fixed Effects variable is declared, the FE Group cell above the inputs selects which group's own average the prediction is anchored to.</t>
+  </si>
+  <si>
+    <t>REGRESSION DIAGNOSTIC GUIDE</t>
+  </si>
+  <si>
+    <t>Use the charts and flagged cells on the Regression sheet to assess model assumptions. Work through Tier 1 first; investigate Tier 2 only when a Tier 1 plot raises a concern.</t>
+  </si>
+  <si>
+    <t>TIER 1 — Review for every model</t>
+  </si>
+  <si>
+    <t>Plot</t>
+  </si>
+  <si>
+    <t>X-axis</t>
+  </si>
+  <si>
+    <t>Y-axis</t>
+  </si>
+  <si>
+    <t>What to look for</t>
+  </si>
+  <si>
+    <t>Residuals vs. Fitted</t>
+  </si>
+  <si>
+    <t>Predicted Y</t>
+  </si>
+  <si>
+    <t>Residuals</t>
+  </si>
+  <si>
+    <t>Random scatter around zero. A curve or funnel shape signals nonlinearity or heteroscedasticity (non-constant error variance).</t>
+  </si>
+  <si>
+    <t>Normal Q-Q</t>
+  </si>
+  <si>
+    <t>Normal Scores (theoretical)</t>
+  </si>
+  <si>
+    <t>Studentized Residuals Ranked</t>
+  </si>
+  <si>
+    <t>Points close to a straight diagonal line. Heavy tails or an S-curve indicate non-normal errors. Check QQ Correlation (Cell P10): below 0.98 = mild concern, below 0.95 = stronger concern.</t>
+  </si>
+  <si>
+    <t>Actual vs. Predicted</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>Points close to a 45° line. A bow or fan shape confirms the same problems seen in Residuals vs. Fitted but from a different angle.</t>
+  </si>
+  <si>
+    <t>TIER 2 — Investigate when Tier 1 raises a concern</t>
+  </si>
+  <si>
+    <t>Scale-Location</t>
+  </si>
+  <si>
+    <t>Scale-Location
+(√|Studentized Residuals|)</t>
+  </si>
+  <si>
+    <t>Flat horizontal spread of points = homoscedasticity. An upward trend confirms heteroscedasticity flagged in Tier 1. Yellow cells: value &gt; √2 ≈ 1.41; red cells: value &gt; √3 ≈ 1.73.</t>
+  </si>
+  <si>
+    <t>Cook's Distance</t>
+  </si>
+  <si>
+    <t>Observation (bar position)</t>
+  </si>
+  <si>
+    <t>Spikes above 4/n (yellow) or above 0.9 (red) mark observations with outsized influence on the fitted coefficients. Bars are ordered by observation number. Inspect those rows for data entry errors or genuine outliers before removing them. Remove outliers only when you have a definitive, non-statistical reason to believe the data point is invalid, comes from a different population, or disproportionately distorts the analysis. Never filter out data solely because it is an extreme statistical value, as doing so can introduce bias and erase genuine insights.</t>
+  </si>
+  <si>
+    <t>Studentized Residuals vs. Leverage</t>
+  </si>
+  <si>
+    <t>Hat Diagonal (leverage)</t>
+  </si>
+  <si>
+    <t>Studentized Residuals</t>
+  </si>
+  <si>
+    <t>High leverage alone is not a problem. Combined high leverage and large residual (top-right or bottom-right of the plot) = influential outlier. Hat &gt; 2p/n is flagged red; Hat &gt; 3p/n is additionally bold.</t>
+  </si>
+  <si>
+    <t>PRESS Residuals</t>
+  </si>
+  <si>
+    <t>PRESS Residual
+(e / (1 − h))</t>
+  </si>
+  <si>
+    <t>PRESS residuals inflate the ordinary residual by leverage. Bars are ordered by observation number. Large values (|PRESS| &gt; 2 × SE yellow, &gt; 3 × SE red) flag observations whose removal would substantially shift the fitted model.</t>
+  </si>
+  <si>
+    <t>DIAGNOSTIC THRESHOLD REFERENCE</t>
+  </si>
+  <si>
+    <t>Diagnostic</t>
+  </si>
+  <si>
+    <t>Location on sheet</t>
+  </si>
+  <si>
+    <t>Yellow threshold</t>
+  </si>
+  <si>
+    <t>Red threshold</t>
+  </si>
+  <si>
+    <t>GVIF (Generalized Variance Inflation Factor)</t>
+  </si>
+  <si>
+    <t>Col U, Predictor Summary</t>
+  </si>
+  <si>
+    <t>GVIF &gt; 5  (possible collinearity)</t>
+  </si>
+  <si>
+    <t>GVIF &gt; 10  (strong collinearity)</t>
+  </si>
+  <si>
+    <t>Tolerance</t>
+  </si>
+  <si>
+    <t>Col V, Predictor Summary</t>
+  </si>
+  <si>
+    <t>Tolerance &lt; 0.2</t>
+  </si>
+  <si>
+    <t>Tolerance &lt; 0.1</t>
+  </si>
+  <si>
+    <t>PRESS R²</t>
+  </si>
+  <si>
+    <t>Cell P5, Diagnostics</t>
+  </si>
+  <si>
+    <t>—</t>
+  </si>
+  <si>
+    <t>PRESS R² &lt; 0  (worse than predicting Y-mean)</t>
+  </si>
+  <si>
+    <t>QQ Correlation</t>
+  </si>
+  <si>
+    <t>Cell P10, Diagnostics</t>
+  </si>
+  <si>
+    <t>&lt; 0.98  (mild non-normality)</t>
+  </si>
+  <si>
+    <t>&lt; 0.95  (clear non-normality)</t>
+  </si>
+  <si>
+    <t>Significance F</t>
+  </si>
+  <si>
+    <t>Cell Q15, ANOVA Table</t>
+  </si>
+  <si>
+    <t>P-value &gt; alpha  (model not significant)</t>
+  </si>
+  <si>
+    <t>Coefficient P-values</t>
+  </si>
+  <si>
+    <t>Col P, Coefficients</t>
+  </si>
+  <si>
+    <t>P-value &gt; alpha  (term not significant)</t>
+  </si>
+  <si>
+    <t>Col AB, Residual Output</t>
+  </si>
+  <si>
+    <t>h &gt; 2p/n  (high leverage)</t>
+  </si>
+  <si>
+    <t>Col AC, Residual Output</t>
+  </si>
+  <si>
+    <t>|r*| &gt; 2  (moderate outlier)</t>
+  </si>
+  <si>
+    <t>|r*| ≥ 3  (strong outlier)</t>
+  </si>
+  <si>
+    <t>Col AD, Residual Output</t>
+  </si>
+  <si>
+    <t>D &gt; 4/n  (review)</t>
+  </si>
+  <si>
+    <t>D &gt; 0.9  (high influence)</t>
+  </si>
+  <si>
+    <t>Col AG, Residual Output</t>
+  </si>
+  <si>
+    <t>&gt; √2 ≈ 1.41  (|r*| &gt; 2 equivalent)</t>
+  </si>
+  <si>
+    <t>&gt; √3 ≈ 1.73  (|r*| &gt; 3 equivalent)</t>
+  </si>
+  <si>
+    <t>PRESS Residual</t>
+  </si>
+  <si>
+    <t>Col AH, Residual Output</t>
+  </si>
+  <si>
+    <t>|PRESS| &gt; 2 × SE</t>
+  </si>
+  <si>
+    <t>|PRESS| &gt; 3 × SE</t>
+  </si>
+  <si>
+    <t>COMMON PATTERNS AND NEXT STEPS</t>
+  </si>
+  <si>
+    <t>Pattern</t>
+  </si>
+  <si>
+    <t>Symptom</t>
+  </si>
+  <si>
+    <t>Next step</t>
+  </si>
+  <si>
+    <t>Heteroscedasticity
+(funnel residuals)</t>
+  </si>
+  <si>
+    <t>Residuals vs. Fitted shows fan shape; Scale-Location trends upward.</t>
+  </si>
+  <si>
+    <t>Consider: log-transforming Y, adding polynomial terms, or fitting a Weighted Least Squares (WLS) model. WLS is planned for a future version of this library.</t>
+  </si>
+  <si>
+    <t>Nonlinearity
+(curved residuals)</t>
+  </si>
+  <si>
+    <t>Residuals vs. Fitted shows a curve; Actual vs. Predicted bows.</t>
+  </si>
+  <si>
+    <t>Add squared or interaction terms to the model. Toggle individual predictors on/off to isolate which variable is driving the curve.</t>
+  </si>
+  <si>
+    <t>Non-normal errors
+(Q-Q deviation)</t>
+  </si>
+  <si>
+    <t>Q-Q plot shows heavy tails or S-curve; QQ Correlation &lt; 0.98.</t>
+  </si>
+  <si>
+    <t>With n &gt; 100 moderate departures rarely invalidate inference. For small n, consider robust standard errors or a bootstrap Confidence Interval approach.</t>
+  </si>
+  <si>
+    <t>Influential observations
+(high Cook's D or PRESS)</t>
+  </si>
+  <si>
+    <t>Cook's D &gt; 4/n or |PRESS| &gt; 2 × SE for one or more rows.</t>
+  </si>
+  <si>
+    <t>Inspect those rows. Verify data entry. Refit without the observation(s) and compare coefficients — if they shift substantially, see which ones and research the reasons why those data points are different. If there's a significant difference, choose one model, but report the prediction results of the other regression as a sensitivity analysis.</t>
+  </si>
+  <si>
+    <t>Multicollinearity
+(high GVIF)</t>
+  </si>
+  <si>
+    <t>GVIF &gt; 10 for one or more predictors. A categorical predictor's dummy columns all show the same shared GVIF value — that's the whole variable's collinearity, not a per-level artifact.</t>
+  </si>
+  <si>
+    <t>Remove or combine correlated predictors. Use the Correlation_Matrix function to identify the pairs. Partial R² shows each predictor's unique contribution after controlling for the others.</t>
+  </si>
+  <si>
     <t>The Variable column fills itself from your table's headers — one specification row per column. For each row, choose a Role:
 Response (y) — the dependent variable; declare exactly one.
 Predictor (x) — a candidate model input; the Include toggle turns it on or off for the current model run.
 Identifier (Row Label) — labeling columns such as names, IDs, or dates; they appear as row labels in the RESIDUAL OUTPUT section (multiple Identifier columns are joined with "|").
 Filter — a TRUE/FALSE or 1/0 column; only rows where every Filter column is truthy enter the regression. Declare several Filter columns to stratify — they are ANDed together.
-Omit — never used for anything; helper columns and notes.</t>
-  </si>
-  <si>
-    <t>For each included Predictor, set its Type. Continuous predictors enter the design matrix as-is. Categorical predictors are dummy-coded automatically: each level except the reference level becomes a 0/1 column with a level-qualified name (e.g. "Status: Developing"). The reference level defaults to the first level in sort order; type a level into Reference Level to override it (the cell turns red if that level does not exist in the analysis sample). The Levels and Reference In Use columns display what the model will do: the distinct level count in the analysis sample, and the reference actually in effect. A categorical with one level (or an invalid reference) is flagged red and contributes no columns — the rest of the model still computes.</t>
-  </si>
-  <si>
-    <t>If your table has more columns than the shipped dataset, fill in Role, Include, and Type for the extra specification rows — the dropdowns are available all the way down. A row with a blank Role is ignored. The Order and Transform columns are placeholders for a future version and are not read by any formula; they are hidden on the sheet. The Sequence column marks at most one variable as the ordering axis for future lag/difference/serial-correlation features — it is independent of Role and Type (a Predictor can also be the sequence axis). Leave it blank for non-panel data; marking two or more rows shows a red error in the status cell above the column. The Sequence Period column (I) is the typed override input: type a number on the flagged row to declare a Δ that differs from the candidate. The Period In Use column (J) is the live companion — it shows the typed override if column I is non-blank, otherwise the computed candidate (the most common gap between consecutive periods within a group). Lag_By and Difference_By fall back to Base_Period_Delta() when their [delta] argument is omitted — never a silent 1.</t>
-  </si>
-  <si>
-    <t>Intercept:</t>
-  </si>
-  <si>
-    <t>The Intercept toggle sits at the top of the Include column (C2). Leave it TRUE for models with Categorical predictors: reference-level dummy coding relies on the intercept to carry the baseline, and the toggle flags red if it is FALSE while a Categorical predictor is included.</t>
-  </si>
-  <si>
-    <t>Which rows are used:</t>
-  </si>
-  <si>
-    <t>The analysis sample is derived automatically — a row is included when the Response is numeric, every included Continuous predictor is numeric, and every Filter column is truthy. There is nothing to configure beyond the Roles. Note that Categorical predictors impose no completeness requirement: rows with a blank category still enter the sample (all of that variable's dummies are blank there) unless a Filter excludes them.</t>
-  </si>
-  <si>
-    <t>Optional — point prediction:</t>
-  </si>
-  <si>
-    <t>Enter a value for each design-matrix column in the orange cells under PREDICTION INPUTS (column AH) — one row per constructed column, including one per dummy (use 1 for the scenario's level, 0 for its siblings; no Intercept row — the model's own baseline is handled automatically). The Training Mean column beside the inputs shows each column's mean over the analysis sample, which is also the prefilled default — so the untouched prediction is at the data's center. Results appear in the PREDICTION OUTPUTS box above as both a mean-response confidence interval (CI) and a wider new-observation prediction interval (PI); the confidence level is controlled by the Alpha cell (Y12) in REGRESSION OUTPUTS. If a Fixed Effects variable is declared, the FE Group cell above the inputs selects which group's own average the prediction is anchored to.</t>
-  </si>
-  <si>
-    <t>REGRESSION DIAGNOSTIC GUIDE</t>
-  </si>
-  <si>
-    <t>Use the charts and flagged cells on the Regression sheet to assess model assumptions. Work through Tier 1 first; investigate Tier 2 only when a Tier 1 plot raises a concern.</t>
-  </si>
-  <si>
-    <t>TIER 1 — Review for every model</t>
-  </si>
-  <si>
-    <t>Plot</t>
-  </si>
-  <si>
-    <t>X-axis</t>
-  </si>
-  <si>
-    <t>Y-axis</t>
-  </si>
-  <si>
-    <t>What to look for</t>
-  </si>
-  <si>
-    <t>Residuals vs. Fitted</t>
-  </si>
-  <si>
-    <t>Predicted Y</t>
-  </si>
-  <si>
-    <t>Residuals</t>
-  </si>
-  <si>
-    <t>Random scatter around zero. A curve or funnel shape signals nonlinearity or heteroscedasticity (non-constant error variance).</t>
-  </si>
-  <si>
-    <t>Normal Q-Q</t>
-  </si>
-  <si>
-    <t>Normal Scores (theoretical)</t>
-  </si>
-  <si>
-    <t>Studentized Residuals Ranked</t>
-  </si>
-  <si>
-    <t>Points close to a straight diagonal line. Heavy tails or an S-curve indicate non-normal errors. Check QQ Correlation (Cell P10): below 0.98 = mild concern, below 0.95 = stronger concern.</t>
-  </si>
-  <si>
-    <t>Actual vs. Predicted</t>
-  </si>
-  <si>
-    <t>Y</t>
-  </si>
-  <si>
-    <t>Points close to a 45° line. A bow or fan shape confirms the same problems seen in Residuals vs. Fitted but from a different angle.</t>
-  </si>
-  <si>
-    <t>TIER 2 — Investigate when Tier 1 raises a concern</t>
-  </si>
-  <si>
-    <t>Scale-Location</t>
-  </si>
-  <si>
-    <t>Scale-Location
-(√|Studentized Residuals|)</t>
-  </si>
-  <si>
-    <t>Flat horizontal spread of points = homoscedasticity. An upward trend confirms heteroscedasticity flagged in Tier 1. Yellow cells: value &gt; √2 ≈ 1.41; red cells: value &gt; √3 ≈ 1.73.</t>
-  </si>
-  <si>
-    <t>Cook's Distance</t>
-  </si>
-  <si>
-    <t>Observation (bar position)</t>
-  </si>
-  <si>
-    <t>Spikes above 4/n (yellow) or above 0.9 (red) mark observations with outsized influence on the fitted coefficients. Bars are ordered by observation number. Inspect those rows for data entry errors or genuine outliers before removing them. Remove outliers only when you have a definitive, non-statistical reason to believe the data point is invalid, comes from a different population, or disproportionately distorts the analysis. Never filter out data solely because it is an extreme statistical value, as doing so can introduce bias and erase genuine insights.</t>
-  </si>
-  <si>
-    <t>Studentized Residuals vs. Leverage</t>
-  </si>
-  <si>
-    <t>Hat Diagonal (leverage)</t>
-  </si>
-  <si>
-    <t>Studentized Residuals</t>
-  </si>
-  <si>
-    <t>High leverage alone is not a problem. Combined high leverage and large residual (top-right or bottom-right of the plot) = influential outlier. Hat &gt; 2p/n is flagged red; Hat &gt; 3p/n is additionally bold.</t>
-  </si>
-  <si>
-    <t>PRESS Residuals</t>
-  </si>
-  <si>
-    <t>PRESS Residual
-(e / (1 − h))</t>
-  </si>
-  <si>
-    <t>PRESS residuals inflate the ordinary residual by leverage. Bars are ordered by observation number. Large values (|PRESS| &gt; 2 × SE yellow, &gt; 3 × SE red) flag observations whose removal would substantially shift the fitted model.</t>
-  </si>
-  <si>
-    <t>DIAGNOSTIC THRESHOLD REFERENCE</t>
-  </si>
-  <si>
-    <t>Diagnostic</t>
-  </si>
-  <si>
-    <t>Location on sheet</t>
-  </si>
-  <si>
-    <t>Yellow threshold</t>
-  </si>
-  <si>
-    <t>Red threshold</t>
-  </si>
-  <si>
-    <t>GVIF (Generalized Variance Inflation Factor)</t>
-  </si>
-  <si>
-    <t>Col U, Predictor Summary</t>
-  </si>
-  <si>
-    <t>GVIF &gt; 5  (possible collinearity)</t>
-  </si>
-  <si>
-    <t>GVIF &gt; 10  (strong collinearity)</t>
-  </si>
-  <si>
-    <t>Tolerance</t>
-  </si>
-  <si>
-    <t>Col V, Predictor Summary</t>
-  </si>
-  <si>
-    <t>Tolerance &lt; 0.2</t>
-  </si>
-  <si>
-    <t>Tolerance &lt; 0.1</t>
-  </si>
-  <si>
-    <t>PRESS R²</t>
-  </si>
-  <si>
-    <t>Cell P5, Diagnostics</t>
-  </si>
-  <si>
-    <t>—</t>
-  </si>
-  <si>
-    <t>PRESS R² &lt; 0  (worse than predicting Y-mean)</t>
-  </si>
-  <si>
-    <t>QQ Correlation</t>
-  </si>
-  <si>
-    <t>Cell P10, Diagnostics</t>
-  </si>
-  <si>
-    <t>&lt; 0.98  (mild non-normality)</t>
-  </si>
-  <si>
-    <t>&lt; 0.95  (clear non-normality)</t>
-  </si>
-  <si>
-    <t>Significance F</t>
-  </si>
-  <si>
-    <t>Cell Q15, ANOVA Table</t>
-  </si>
-  <si>
-    <t>P-value &gt; alpha  (model not significant)</t>
-  </si>
-  <si>
-    <t>Coefficient P-values</t>
-  </si>
-  <si>
-    <t>Col P, Coefficients</t>
-  </si>
-  <si>
-    <t>P-value &gt; alpha  (term not significant)</t>
-  </si>
-  <si>
-    <t>Col AB, Residual Output</t>
-  </si>
-  <si>
-    <t>h &gt; 2p/n  (high leverage)</t>
-  </si>
-  <si>
-    <t>Col AC, Residual Output</t>
-  </si>
-  <si>
-    <t>|r*| &gt; 2  (moderate outlier)</t>
-  </si>
-  <si>
-    <t>|r*| ≥ 3  (strong outlier)</t>
-  </si>
-  <si>
-    <t>Col AD, Residual Output</t>
-  </si>
-  <si>
-    <t>D &gt; 4/n  (review)</t>
-  </si>
-  <si>
-    <t>D &gt; 0.9  (high influence)</t>
-  </si>
-  <si>
-    <t>Col AG, Residual Output</t>
-  </si>
-  <si>
-    <t>&gt; √2 ≈ 1.41  (|r*| &gt; 2 equivalent)</t>
-  </si>
-  <si>
-    <t>&gt; √3 ≈ 1.73  (|r*| &gt; 3 equivalent)</t>
-  </si>
-  <si>
-    <t>PRESS Residual</t>
-  </si>
-  <si>
-    <t>Col AH, Residual Output</t>
-  </si>
-  <si>
-    <t>|PRESS| &gt; 2 × SE</t>
-  </si>
-  <si>
-    <t>|PRESS| &gt; 3 × SE</t>
-  </si>
-  <si>
-    <t>COMMON PATTERNS AND NEXT STEPS</t>
-  </si>
-  <si>
-    <t>Pattern</t>
-  </si>
-  <si>
-    <t>Symptom</t>
-  </si>
-  <si>
-    <t>Next step</t>
-  </si>
-  <si>
-    <t>Heteroscedasticity
-(funnel residuals)</t>
-  </si>
-  <si>
-    <t>Residuals vs. Fitted shows fan shape; Scale-Location trends upward.</t>
-  </si>
-  <si>
-    <t>Consider: log-transforming Y, adding polynomial terms, or fitting a Weighted Least Squares (WLS) model. WLS is planned for a future version of this library.</t>
-  </si>
-  <si>
-    <t>Nonlinearity
-(curved residuals)</t>
-  </si>
-  <si>
-    <t>Residuals vs. Fitted shows a curve; Actual vs. Predicted bows.</t>
-  </si>
-  <si>
-    <t>Add squared or interaction terms to the model. Toggle individual predictors on/off to isolate which variable is driving the curve.</t>
-  </si>
-  <si>
-    <t>Non-normal errors
-(Q-Q deviation)</t>
-  </si>
-  <si>
-    <t>Q-Q plot shows heavy tails or S-curve; QQ Correlation &lt; 0.98.</t>
-  </si>
-  <si>
-    <t>With n &gt; 100 moderate departures rarely invalidate inference. For small n, consider robust standard errors or a bootstrap Confidence Interval approach.</t>
-  </si>
-  <si>
-    <t>Influential observations
-(high Cook's D or PRESS)</t>
-  </si>
-  <si>
-    <t>Cook's D &gt; 4/n or |PRESS| &gt; 2 × SE for one or more rows.</t>
-  </si>
-  <si>
-    <t>Inspect those rows. Verify data entry. Refit without the observation(s) and compare coefficients — if they shift substantially, see which ones and research the reasons why those data points are different. If there's a significant difference, choose one model, but report the prediction results of the other regression as a sensitivity analysis.</t>
-  </si>
-  <si>
-    <t>Multicollinearity
-(high GVIF)</t>
-  </si>
-  <si>
-    <t>GVIF &gt; 10 for one or more predictors. A categorical predictor's dummy columns all show the same shared GVIF value — that's the whole variable's collinearity, not a per-level artifact.</t>
-  </si>
-  <si>
-    <t>Remove or combine correlated predictors. Use the Correlation_Matrix function to identify the pairs. Partial R² shows each predictor's unique contribution after controlling for the others.</t>
+Omit — never used for anything; helper columns and notes.
+Fixed Effects — declare exactly one panel-grouping variable; the model absorbs a separate intercept per group (one-way within transformation) instead of pooled OLS, crediting the absorbed degrees of freedom back into inference. Type and Reference Level don't apply to this row — leave them as-is.</t>
   </si>
 </sst>
 </file>
@@ -810,49 +811,49 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:1" ht="135" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:1" ht="180" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>6</v>
+        <v>107</v>
       </c>
     </row>
     <row r="10" spans="1:1" ht="90" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11" spans="1:1" ht="150" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14" spans="1:1" ht="45" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17" spans="1:1" ht="60" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="20" spans="1:1" ht="120" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -872,7 +873,7 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -880,12 +881,12 @@
     </row>
     <row r="2" spans="1:4" ht="90" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B4" s="5"/>
       <c r="C4" s="5"/>
@@ -893,63 +894,63 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="C5" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="D5" s="4" t="s">
         <v>20</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C6" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="D6" s="2" t="s">
         <v>24</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="C7" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="D7" s="2" t="s">
         <v>28</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C8" s="2" t="s">
+      <c r="D8" s="2" t="s">
         <v>31</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
@@ -957,77 +958,77 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="C11" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="D11" s="4" t="s">
         <v>20</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B12" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C12" s="2" t="s">
+      <c r="D12" s="2" t="s">
         <v>35</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="180" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="C13" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D13" s="2" t="s">
         <v>38</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="C14" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="D14" s="2" t="s">
         <v>42</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="75" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B15" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C15" s="2" t="s">
+      <c r="D15" s="2" t="s">
         <v>45</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B17" s="5"/>
       <c r="C17" s="5"/>
@@ -1035,243 +1036,243 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B18" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="C18" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="D18" s="4" t="s">
         <v>50</v>
-      </c>
-      <c r="D18" s="4" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B19" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="C19" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="D19" s="2" t="s">
         <v>54</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B20" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="C20" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="D20" s="2" t="s">
         <v>58</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B21" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="C21" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="D21" s="2" t="s">
         <v>62</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B22" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="C22" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="D22" s="2" t="s">
         <v>66</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B23" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="C23" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="D23" s="2" t="s">
         <v>69</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B24" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="C24" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="D24" s="2" t="s">
         <v>72</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B25" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="D25" s="2" t="s">
         <v>74</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B26" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C26" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="C26" s="2" t="s">
+      <c r="D26" s="2" t="s">
         <v>77</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B27" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C27" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="C27" s="2" t="s">
+      <c r="D27" s="2" t="s">
         <v>80</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B28" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C28" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="C28" s="2" t="s">
+      <c r="D28" s="2" t="s">
         <v>83</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B29" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="B29" s="2" t="s">
+      <c r="C29" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="C29" s="2" t="s">
+      <c r="D29" s="2" t="s">
         <v>87</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B31" s="5"/>
       <c r="C31" s="5"/>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="B32" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="B32" s="4" t="s">
+      <c r="C32" s="4" t="s">
         <v>91</v>
-      </c>
-      <c r="C32" s="4" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="120" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B33" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="B33" s="2" t="s">
+      <c r="C33" s="2" t="s">
         <v>94</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="105" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="B34" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="B34" s="2" t="s">
+      <c r="C34" s="2" t="s">
         <v>97</v>
-      </c>
-      <c r="C34" s="2" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="120" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B35" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="B35" s="2" t="s">
+      <c r="C35" s="2" t="s">
         <v>100</v>
-      </c>
-      <c r="C35" s="2" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="240" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="B36" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="B36" s="2" t="s">
+      <c r="C36" s="2" t="s">
         <v>103</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="37" spans="1:3" ht="150" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B37" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="B37" s="2" t="s">
+      <c r="C37" s="2" t="s">
         <v>106</v>
-      </c>
-      <c r="C37" s="2" t="s">
-        <v>107</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Enhance regression sheet functionality and testing
- Updated static sheets with new data.
- Added new expected case names in regression tests.
- Introduced new constants for sheet writing and updated related tests.
- Implemented unit space block writing in regression output tests.
- Updated version history to reflect the new version 3.3.0.
- Enhanced regression sheet inspection to handle precision issues in comparisons.
- Added comprehensive tests for unit space dispatch functions, ensuring correctness against OLS reference.
</commit_message>
<xml_diff>
--- a/templates/static_sheets.xlsx
+++ b/templates/static_sheets.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Stephen_Colodner\windows code\Statistical_Analysis_Lambda_Catalog\.claude\worktrees\3-0-changeover-stage-3-263d53\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Stephen_Colodner\windows code\Statistical_Analysis_Lambda_Catalog\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7C3CE199-38F8-42C4-B598-08D44514720F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{59ADFA01-E38B-4F00-B7B0-532E4364F778}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{1411C739-6A2D-448E-B19F-D2DD9A0E5CC5}"/>
   </bookViews>
@@ -373,10 +373,10 @@
     <t>Define your model in the MODEL SPECIFICATION block (columns A–O):</t>
   </si>
   <si>
-    <t>If your table has more columns than the shipped dataset, fill in Role, Include, and Type for the extra specification rows — the dropdowns are available all the way down. A row with a blank Role is ignored. The Order column is a placeholder for a future version and is not read by any formula; it is hidden on the sheet. The Transform column offers Log on the Response row and on Continuous Predictor rows: the model fits in natural-log space for that variable, and affected outputs are labeled "(Log)" — results are not converted back to raw units. Log is not valid on a Categorical Predictor; setting it there flags the cell red and the fit still runs with that row's Transform ignored (dummy-coded as usual). The Sequence column marks at most one variable as the ordering axis for future lag/difference/serial-correlation features — it is independent of Role and Type (a Predictor can also be the sequence axis). Leave it blank for non-panel data; marking two or more rows shows a red error in the status cell above the column. The Sequence Period column (I) is the typed override input: type a number on the flagged row to declare a Δ that differs from the candidate. The Period In Use column (J) is the live companion — it shows the typed override if column I is non-blank, otherwise the computed candidate (the most common gap between consecutive periods within a group). Lag_By and Difference_By fall back to Base_Period_Delta() when their [delta] argument is omitted — never a silent 1. The Interaction Term (M) and Interaction Operation (N) columns declare an interaction between this row and another Predictor — pick the other variable and one of Product, Difference, or Ratio. They are placeholders in this release: the dropdowns, the marginality warning (amber when the named Predictor is excluded), and the duplicate-column error (red when two rows declare the same symmetric interaction of each other) are all live, but no constructor builds the columns yet. The Design Columns column (O) shows how many design-matrix columns each row contributes — 1 for a Continuous predictor, one less than the Levels count for a Categorical one. The total above it, with the intercept added, is the full width of the constructed design matrix; it turns amber on a model wide enough to be slow and red on one too wide for the sheet.</t>
-  </si>
-  <si>
     <t>Enter a value for each design-matrix column in the orange cells under PREDICTION INPUTS (column AK) — one row per constructed column, including one per dummy (use 1 for the scenario's level, 0 for its siblings; no Intercept row — the model's own baseline is handled automatically). The Training Mean column beside the inputs shows each column's mean over the analysis sample, which is also the prefilled default — so the untouched prediction is at the data's center. Results appear in the PREDICTION OUTPUTS box above as both a mean-response confidence interval (CI) and a wider new-observation prediction interval (PI); the confidence level is controlled by the Alpha cell (AB12) in REGRESSION OUTPUTS. If a Fixed Effects variable is declared, the FE Group cell above the inputs selects which group's own average the prediction is anchored to.</t>
+  </si>
+  <si>
+    <t>If your table has more columns than the shipped dataset, fill in Role, Include, and Type for the extra specification rows — the dropdowns are available all the way down. A row with a blank Role is ignored. The Order column is a placeholder for a future version and is not read by any formula; it is hidden on the sheet. The Transform column offers Log on the Response row and on Continuous Predictor rows: the model fits in natural-log space for that variable, and affected outputs are labeled "(Log)" — but the Unit-Space Fit block at AG3:AH9 reports the back-transformed R² / Adj R² / RMSE in original units (Duan smearing by default, Naive on the AH4 toggle), and the Prediction Outputs block's Original Units column (AL) carries the back-transformed point estimate and the four CI/PI bounds. The two new Residual Output columns (AZ, BA) carry Predicted Y and Residual in original units. Under Log, the Duan point estimate does not sit at the centre of the four Naive CI/PI bounds (the conditional mean is offset from the conditional median). Log is not valid on a Categorical Predictor; setting it there flags the cell red and the fit still runs with that row's Transform ignored (dummy-coded as usual). The Sequence column marks at most one variable as the ordering axis for future lag/difference/serial-correlation features — it is independent of Role and Type (a Predictor can also be the sequence axis). Leave it blank for non-panel data; marking two or more rows shows a red error in the status cell above the column. The Sequence Period column (I) is the typed override input: type a number on the flagged row to declare a Δ that differs from the candidate. The Period In Use column (J) is the live companion — it shows the typed override if column I is non-blank, otherwise the computed candidate (the most common gap between consecutive periods within a group). Lag_By and Difference_By fall back to Base_Period_Delta() when their [delta] argument is omitted — never a silent 1. The Interaction Term (M) and Interaction Operation (N) columns declare an interaction between this row and another Predictor — pick the other variable and one of Product, Difference, or Ratio. They are placeholders in this release: the dropdowns, the marginality warning (amber when the named Predictor is excluded), and the duplicate-column error (red when two rows declare the same symmetric interaction of each other) are all live, but no constructor builds the columns yet. The Design Columns column (O) shows how many design-matrix columns each row contributes — 1 for a Continuous predictor, one less than the Levels count for a Categorical one. The total above it, with the intercept added, is the full width of the constructed design matrix; it turns amber on a model wide enough to be slow and red on one too wide for the sheet.</t>
   </si>
 </sst>
 </file>
@@ -821,9 +821,9 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:1" ht="300" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:1" ht="360" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
@@ -853,7 +853,7 @@
     </row>
     <row r="20" spans="1:1" ht="120" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update test sheet writers to fix CI errors. Upload error logs. Rebuild dists and the static sheets.
</commit_message>
<xml_diff>
--- a/templates/static_sheets.xlsx
+++ b/templates/static_sheets.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Stephen_Colodner\windows code\Statistical_Analysis_Lambda_Catalog\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\local_python\Statistical_Analysis_Lambda_Catalog\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EEA7A817-D997-4774-BCA8-EAF20A08EF36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4FEBC25A-861C-407D-A72E-8BD6708F4DDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{1411C739-6A2D-448E-B19F-D2DD9A0E5CC5}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{1411C739-6A2D-448E-B19F-D2DD9A0E5CC5}"/>
   </bookViews>
   <sheets>
     <sheet name="Regression Instructions" sheetId="2" r:id="rId1"/>

</xml_diff>

<commit_message>
Update static_sheets.xlsx with new data and formatting changes
</commit_message>
<xml_diff>
--- a/templates/static_sheets.xlsx
+++ b/templates/static_sheets.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Stephen_Colodner\windows code\Statistical_Analysis_Lambda_Catalog\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AF1288E7-5987-4580-AA2A-95E8B54AEAFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7A0C5438-B4BF-49C3-BE62-93CA8175CDE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{1411C739-6A2D-448E-B19F-D2DD9A0E5CC5}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="109">
   <si>
     <t>How to use the Regression sheet for Multilinear Regression (MLR)</t>
   </si>
@@ -245,39 +245,18 @@
     <t>Coefficient P-values</t>
   </si>
   <si>
-    <t>Col P, Coefficients</t>
-  </si>
-  <si>
     <t>P-value &gt; alpha  (term not significant)</t>
   </si>
   <si>
-    <t>Col AB, Residual Output</t>
-  </si>
-  <si>
     <t>h &gt; 2p/n  (high leverage)</t>
   </si>
   <si>
-    <t>Col AC, Residual Output</t>
-  </si>
-  <si>
     <t>|r*| &gt; 2  (moderate outlier)</t>
   </si>
   <si>
     <t>|r*| ≥ 3  (strong outlier)</t>
   </si>
   <si>
-    <t>Col AD, Residual Output</t>
-  </si>
-  <si>
-    <t>D &gt; 4/n  (review)</t>
-  </si>
-  <si>
-    <t>D &gt; 0.9  (high influence)</t>
-  </si>
-  <si>
-    <t>Col AG, Residual Output</t>
-  </si>
-  <si>
     <t>&gt; √2 ≈ 1.41  (|r*| &gt; 2 equivalent)</t>
   </si>
   <si>
@@ -285,9 +264,6 @@
   </si>
   <si>
     <t>PRESS Residual</t>
-  </si>
-  <si>
-    <t>Col AH, Residual Output</t>
   </si>
   <si>
     <t>|PRESS| &gt; 2 × SE</t>
@@ -383,6 +359,27 @@
   </si>
   <si>
     <t>Open the Name Manager (Formulas → Name Manager) and update Source_Table (the "Refers To" field) to your table, including its header row — for example =MyTable[#All]. Everything else derives from this one name: the header row, the data body, and the variable list in the MODEL SPECIFICATION block all update automatically. Source_Table points at LifeExpectancyData by default (a curated four-driver Life Expectancy model — Adult Mortality, Alcohol, percentage expenditure, and Status); a second sample table, MileageData (on the Mileage Data sheet), ships with the workbook for a multi-level categorical-encoding demo (MPG ~ Horsepower + Weight + C(Model Year) + C(Origin) — reach it with --regression-dataset auto_mpg). Practice the retarget on either before pointing at your own data.</t>
+  </si>
+  <si>
+    <t>Col AE, Coefficients</t>
+  </si>
+  <si>
+    <t>Col AR, Residual Output</t>
+  </si>
+  <si>
+    <t>Col AS, Residual Output</t>
+  </si>
+  <si>
+    <t>Col AT, Residual Output</t>
+  </si>
+  <si>
+    <t>D &gt; F.INV(0.5, p, n-p)  (high influence)</t>
+  </si>
+  <si>
+    <t>Col AW, Residual Output</t>
+  </si>
+  <si>
+    <t>Col AX, Residual Output</t>
   </si>
 </sst>
 </file>
@@ -809,17 +806,17 @@
     </row>
     <row r="6" spans="1:1" ht="105" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
     </row>
     <row r="9" spans="1:1" ht="180" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
     </row>
     <row r="10" spans="1:1" ht="90" x14ac:dyDescent="0.25">
@@ -829,7 +826,7 @@
     </row>
     <row r="11" spans="1:1" ht="360" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
@@ -859,17 +856,17 @@
     </row>
     <row r="20" spans="1:1" ht="120" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
     </row>
     <row r="23" spans="1:1" ht="120" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -1139,13 +1136,13 @@
         <v>66</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>67</v>
+        <v>102</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>57</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
@@ -1153,13 +1150,13 @@
         <v>36</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>69</v>
+        <v>103</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>57</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -1167,13 +1164,13 @@
         <v>37</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>71</v>
+        <v>104</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
@@ -1181,13 +1178,13 @@
         <v>32</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>74</v>
+        <v>105</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>75</v>
+        <v>57</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>76</v>
+        <v>106</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -1195,100 +1192,100 @@
         <v>29</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>77</v>
+        <v>107</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>81</v>
+        <v>108</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="B31" s="5"/>
       <c r="C31" s="5"/>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="120" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="105" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="120" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="240" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
     </row>
     <row r="37" spans="1:3" ht="150" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix stale interaction text and add chart-title notes to static reference sheets
- Regression Instructions: replace the false "placeholders, no constructor
  builds the columns" claim in row 11 (interactions shipped in v3.1) and
  correct the Alpha cite AB12 -> AB13
- Modeling Concepts: rename column 2 to "What Problem It Solves", reorder
  features simple-to-complex, append a PLANNED FEATURES section
  (Weight/WLS v3.7, Cluster v3.5, Time v3.6, Two-way FE v3.8, Order col F)
- Diagnostic Guide: document the live-stat chart-title integrations
  (Q-Q r, Adj R2, mean leverage, Cook's cutoff, PRESS total) and add the
  threshold-table footnote (thresholds surface in three places)
- Present-tense fix for the stale RESERVED-and-unwired comments in
  write_spec_block.py / spec_layout.py; Diagnostic Guide docstring now
  points at scripts/rebuild_static_sheets.py

Template regenerated, dist rebuilt and verified; poe verify-models 33/33.

Co-Authored-By: Claude Code <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/static_sheets.xlsx
+++ b/templates/static_sheets.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Stephen_Colodner\windows_code\Statistical_Analysis_Lambda_Catalog\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{56BB81F4-176B-4944-B5A9-5455F91C379C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C2497202-977F-46D5-92AA-70C3C8E3310D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3465" yWindow="3465" windowWidth="21600" windowHeight="11295" activeTab="2" xr2:uid="{1411C739-6A2D-448E-B19F-D2DD9A0E5CC5}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="166">
   <si>
     <t>How to use the Regression sheet for Multilinear Regression (MLR)</t>
   </si>
@@ -76,9 +76,6 @@
     <t>REGRESSION DIAGNOSTIC GUIDE</t>
   </si>
   <si>
-    <t>Use the charts and flagged cells on the Regression sheet to assess model assumptions. Work through Tier 1 first; investigate Tier 2 only when a Tier 1 plot raises a concern.</t>
-  </si>
-  <si>
     <t>TIER 1 — Review for every model</t>
   </si>
   <si>
@@ -115,16 +112,10 @@
     <t>Studentized Residuals Ranked</t>
   </si>
   <si>
-    <t>Points close to a straight diagonal line. Heavy tails or an S-curve indicate non-normal errors. Check QQ Correlation (Cell P10): below 0.98 = mild concern, below 0.95 = stronger concern.</t>
-  </si>
-  <si>
     <t>Actual vs. Predicted</t>
   </si>
   <si>
     <t>Y</t>
-  </si>
-  <si>
-    <t>Points close to a 45° line. A bow or fan shape confirms the same problems seen in Residuals vs. Fitted but from a different angle.</t>
   </si>
   <si>
     <t>TIER 2 — Investigate when Tier 1 raises a concern</t>
@@ -155,17 +146,11 @@
     <t>Studentized Residuals</t>
   </si>
   <si>
-    <t>High leverage alone is not a problem. Combined high leverage and large residual (top-right or bottom-right of the plot) = influential outlier. Hat &gt; 2p/n is flagged red; Hat &gt; 3p/n is additionally bold.</t>
-  </si>
-  <si>
     <t>PRESS Residuals</t>
   </si>
   <si>
     <t>PRESS Residual
 (e / (1 − h))</t>
-  </si>
-  <si>
-    <t>PRESS residuals inflate the ordinary residual by leverage. Bars are ordered by observation number. Large values (|PRESS| &gt; 2 × SE yellow, &gt; 3 × SE red) flag observations whose removal would substantially shift the fitted model.</t>
   </si>
   <si>
     <t>DIAGNOSTIC THRESHOLD REFERENCE</t>
@@ -341,9 +326,6 @@
     <t>Define your model in the MODEL SPECIFICATION block (columns A–O):</t>
   </si>
   <si>
-    <t>Enter a value for each design-matrix column in the orange cells under PREDICTION INPUTS (column AK) — one row per constructed column, including one per dummy (use 1 for the scenario's level, 0 for its siblings; no Intercept row — the model's own baseline is handled automatically). The Training Mean column beside the inputs shows each column's mean over the analysis sample, which is also the prefilled default — so the untouched prediction is at the data's center. Results appear in the PREDICTION OUTPUTS box above as both a mean-response confidence interval (CI) and a wider new-observation prediction interval (PI); the confidence level is controlled by the Alpha cell (AB12) in REGRESSION OUTPUTS. If a Fixed Effects variable is declared, the FE Group cell above the inputs selects which group's own average the prediction is anchored to.</t>
-  </si>
-  <si>
     <t>Optional – faster charts on a fixed-size dataset:</t>
   </si>
   <si>
@@ -371,28 +353,16 @@
     <t>Col AX, Residual Output</t>
   </si>
   <si>
-    <t>If your table has more columns than the shipped dataset, fill in Role, Include, and Type for the extra specification rows — the dropdowns are available all the way down. A row with a blank Role is ignored. The Order column is a placeholder for a future version and is not read by any formula; it is hidden on the sheet. The Transform column offers Log on the Response row and on Continuous Predictor rows: the model fits in natural-log space for that variable, and affected outputs are labeled "(Log)" — but the Unit-Space Fit block at AG4:AH10 reports the back-transformed R² / Adj R² / RMSE in original units (Duan smearing by default, Naive on the AH5 toggle), and the Prediction Outputs block's Original Units column (AL) carries the back-transformed point estimate and the four CI/PI bounds. The two new Residual Output columns (AZ, BA) carry Predicted Y and Residual in original units. Under Log, the Duan point estimate does not sit at the centre of the four Naive CI/PI bounds (the conditional mean is offset from the conditional median). Log is not valid on a Categorical Predictor; setting it there flags the cell red and the fit still runs with that row's Transform ignored (dummy-coded as usual). The Sequence column marks at most one variable as the ordering axis for future lag/difference/serial-correlation features — it is independent of Role and Type (a Predictor can also be the sequence axis). Leave it blank for non-panel data; marking two or more rows shows a red error in the status cell above the column. The Sequence Period column (I) is the typed override input: type a number on the flagged row to declare a Δ that differs from the candidate. The Period In Use column (J) is the live companion — it shows the typed override if column I is non-blank, otherwise the computed candidate (the most common gap between consecutive periods within a group). Lag_By and Difference_By fall back to Base_Period_Delta() when their [delta] argument is omitted — never a silent 1. The Interaction Term (M) and Interaction Operation (N) columns declare an interaction between this row and another Predictor — pick the other variable and one of Product, Difference, or Ratio. They are placeholders in this release: the dropdowns, the marginality warning (amber when the named Predictor is excluded), and the duplicate-column error (red when two rows declare the same symmetric interaction of each other) are all live, but no constructor builds the columns yet. The Design Columns column (O) shows how many design-matrix columns each row contributes — 1 for a Continuous predictor, one less than the Levels count for a Categorical one. The total above it, with the intercept added, is the full width of the constructed design matrix; it turns amber on a model wide enough to be slow and red on one too wide for the sheet.</t>
-  </si>
-  <si>
     <t>The seven diagnostic charts read each series from a worksheet-scoped named range (the RegChart* names) built with OFFSET and sized to the live observation count at $AB$9. OFFSET is volatile, so those ranges re-evaluate on every recalculation pass. If your dataset size is stable, you can remove that overhead by pointing each chart series directly at the absolute range the name resolves to — from row 4 (one below the column header) down to row 3+N, where N is the count shown at $AB$9 (for 200 observations, for example ='Regression'!$AP$4:$AP$203). Select the chart, click a series, and replace the ='Regression'!RegChart... reference in the formula bar with the absolute range. The trade-off is that the chart no longer resizes if you add or drop rows — you must re-point it when the row count changes. The named ranges can stay defined; there is no need to delete them.</t>
   </si>
   <si>
-    <t>Spikes above F.INV(0.5, p, n-p) — the median of the reference F distribution, so the bar to beat scales with the model's own size — mark observations with outsized influence on the fitted coefficients. Bars are ordered by observation number. Inspect those rows for data entry errors or genuine outliers before removing them. Remove outliers only when you have a definitive, non-statistical reason to believe the data point is invalid, comes from a different population, or disproportionately distorts the analysis. Never filter out data solely because it is an extreme statistical value, as doing so can introduce bias and erase genuine insights.</t>
-  </si>
-  <si>
     <t>Cook's D &gt; F.INV(0.5, p, n-p) or |PRESS| &gt; 2 × SE for one or more rows.</t>
   </si>
   <si>
     <t>MODELING CONCEPTS — THE WHY BEHIND EACH FEATURE</t>
   </si>
   <si>
-    <t>Each feature on the Regression sheet exists to make a specific statistical method available without formulas or add-ins. This table explains that link: the point of the feature, the method it enables, and a concrete situation for using it. For the mechanics of setting a feature up, see the Regression Instructions sheet; for how to read the fitted model's residual plots, see the Diagnostic Guide.</t>
-  </si>
-  <si>
     <t>Feature</t>
-  </si>
-  <si>
-    <t>The Point</t>
   </si>
   <si>
     <t>Statistical Method</t>
@@ -490,6 +460,115 @@
   </si>
   <si>
     <t>Theory says cost is zero at zero production, or the instrument reads zero with no input? Turn the intercept off for a regression-through-origin fit. Otherwise leave it on and let it absorb the reference levels' baseline.</t>
+  </si>
+  <si>
+    <t>If your table has more columns than the shipped dataset, fill in Role, Include, and Type for the extra specification rows — the dropdowns are available all the way down. A row with a blank Role is ignored. The Order column is a placeholder for a future version and is not read by any formula; it is hidden on the sheet. The Transform column offers Log on the Response row and on Continuous Predictor rows: the model fits in natural-log space for that variable, and affected outputs are labeled "(Log)" — but the Unit-Space Fit block at AG4:AH10 reports the back-transformed R² / Adj R² / RMSE in original units (Duan smearing by default, Naive on the AH5 toggle), and the Prediction Outputs block's Original Units column (AL) carries the back-transformed point estimate and the four CI/PI bounds. The two new Residual Output columns (AZ, BA) carry Predicted Y and Residual in original units. Under Log, the Duan point estimate does not sit at the centre of the four Naive CI/PI bounds (the conditional mean is offset from the conditional median). Log is not valid on a Categorical Predictor; setting it there flags the cell red and the fit still runs with that row's Transform ignored (dummy-coded as usual). The Sequence column marks at most one variable as the ordering axis for future lag/difference/serial-correlation features — it is independent of Role and Type (a Predictor can also be the sequence axis). Leave it blank for non-panel data; marking two or more rows shows a red error in the status cell above the column. The Sequence Period column (I) is the typed override input: type a number on the flagged row to declare a Δ that differs from the candidate. The Period In Use column (J) is the live companion — it shows the typed override if column I is non-blank, otherwise the computed candidate (the most common gap between consecutive periods within a group). Lag_By and Difference_By fall back to Base_Period_Delta() when their [delta] argument is omitted — never a silent 1. The Interaction Term (M) and Interaction Operation (N) columns declare an interaction between this row and another Predictor — pick the other variable and one of Product, Difference, or Ratio. The interaction column is built into the design matrix automatically: Continuous × Continuous adds 1 column, Continuous × Categorical adds one per retained level, and Categorical × Categorical adds the full product of the two. Naming this row's own variable with Operation = Product is the documented way to declare a quadratic (x²) term. An interaction whose mate is switched off (Include = FALSE) still builds and is flagged amber as a marginality warning; a reciprocal declaration — two rows naming each other under Product or Difference — is flagged red, because it would duplicate or negate a column and make the matrix singular. Interaction rows also appear in PREDICTION INPUTS; leave them at the Training Mean defaults or type scenario values. The Design Columns column (O) shows how many design-matrix columns each row contributes — 1 for a Continuous predictor, one less than the Levels count for a Categorical one. The total above it, with the intercept added, is the full width of the constructed design matrix; it turns amber on a model wide enough to be slow and red on one too wide for the sheet.</t>
+  </si>
+  <si>
+    <t>Enter a value for each design-matrix column in the orange cells under PREDICTION INPUTS (column AK) — one row per constructed column, including one per dummy (use 1 for the scenario's level, 0 for its siblings; no Intercept row — the model's own baseline is handled automatically). The Training Mean column beside the inputs shows each column's mean over the analysis sample, which is also the prefilled default — so the untouched prediction is at the data's center. Results appear in the PREDICTION OUTPUTS box above as both a mean-response confidence interval (CI) and a wider new-observation prediction interval (PI); the confidence level is controlled by the Alpha cell (AB13) in REGRESSION OUTPUTS. If a Fixed Effects variable is declared, the FE Group cell above the inputs selects which group's own average the prediction is anchored to.</t>
+  </si>
+  <si>
+    <t>Each feature on the Regression sheet exists to make a specific statistical method available without formulas or add-ins. This table explains that link: what problem the feature solves, the method it enables, and a concrete situation for using it. For the mechanics of setting a feature up, see the Regression Instructions sheet; for how to read the fitted model's residual plots, see the Diagnostic Guide.</t>
+  </si>
+  <si>
+    <t>What Problem It Solves</t>
+  </si>
+  <si>
+    <t>PLANNED FEATURES — DECLARED IN THE SHEET, NOT YET BUILT</t>
+  </si>
+  <si>
+    <t>The features below are declared in the sheet's structure — a Role value in the dropdown, a reserved column — but no formula builds them in this release. Each row states what problem the feature will solve when it ships, and what to use in the meantime.</t>
+  </si>
+  <si>
+    <t>Weight — WLS
+(Role = Weight, v3.7)
+PLANNED, future release</t>
+  </si>
+  <si>
+    <t>Some observations are known to be noisier than others — each row averages a different number of underlying readings, or a variance you can quantify at row level. OLS gives the noisy rows the same vote as the precise ones.</t>
+  </si>
+  <si>
+    <t>Weighted Least Squares: each row enters the fit scaled by its known variance, so precise observations dominate. The Weight Role will name the column carrying that variance.</t>
+  </si>
+  <si>
+    <t>Today's workaround is the Diagnostic Guide's heteroscedasticity guidance: a Log transform on the response, or an interaction / quadratic term when the variance tracks a predictor's mean.</t>
+  </si>
+  <si>
+    <t>Cluster
+(Role = Cluster, v3.5)
+PLANNED, future release</t>
+  </si>
+  <si>
+    <t>Rows collected in groups — plants, firms, countries — share unmodeled shocks, so nominally-independent standard errors are too optimistic (they overstate significance).</t>
+  </si>
+  <si>
+    <t>Clustered-robust variance estimator: the same coefficients, with standard errors that allow arbitrary correlation within a group. Partially forward-wired — the Role slot and a dormant branch in Serial_Correlation_Group() await the estimator.</t>
+  </si>
+  <si>
+    <t>Survey or panel data where rows within one cluster move together: name the cluster column and the P-values and confidence intervals stop assuming every row is independent.</t>
+  </si>
+  <si>
+    <t>Time
+(Role = Time, v3.6)
+PLANNED, future release</t>
+  </si>
+  <si>
+    <t>A panel needs an explicit time index distinct from 'which group a row belongs to' — lag and difference features must follow time within a unit, not sheet order.</t>
+  </si>
+  <si>
+    <t>Time-index designation: the Role names the column holding each row's time value; Lag_By / Difference_By and the future Time Series sheet are its consumers. The Role ships first, the sheet last.</t>
+  </si>
+  <si>
+    <t>Until then, the Sequence flag (column H) plus its Sequence Period override already carries the ordering axis for the shipped lag/difference features.</t>
+  </si>
+  <si>
+    <t>Two-way Fixed Effects
+(v3.8)
+PLANNED, future release</t>
+  </si>
+  <si>
+    <t>Sometimes the stable nuisance is two-dimensional — both the plant AND the year leave a fixed mark on every observation, and absorbing only one of them leaves the other confounding the coefficients.</t>
+  </si>
+  <si>
+    <t>Absorb_Two_Way_Fixed_Effects: the within transformation applied along two group axes at once. Today at most ONE Fixed Effects row is legal — two or more is a red spec error, by design, until this lands.</t>
+  </si>
+  <si>
+    <t>Plant-and-year panels: for now, keep one Fixed Effects row and use a Filter to narrow the sample, or dummy-code the second axis as a Categorical predictor.</t>
+  </si>
+  <si>
+    <t>Order
+(column F)
+PLANNED, future release</t>
+  </si>
+  <si>
+    <t>Term order in the coefficient table currently follows the source table's column order — fine for every model so far, but a hand-authored spec may want terms presented in a chosen sequence.</t>
+  </si>
+  <si>
+    <t>A reserved, hidden column (width 0): it will control each spec row's position in the constructed design matrix and the coefficient table. No formula reads it in this release.</t>
+  </si>
+  <si>
+    <t>Nothing to do today — the column is hidden and ignored; leave it blank if you reveal it.</t>
+  </si>
+  <si>
+    <t>Use the charts and flagged cells on the Regression sheet to assess model assumptions. Work through Tier 1 first; investigate Tier 2 only when a Tier 1 plot raises a concern. Each chart's title carries the live statistics it judges against — the Q-Q correlation, the Adjusted R², the mean leverage, the Cook's Distance cutoff and the PRESS total — so a chart can be read without scrolling back to its source cell.</t>
+  </si>
+  <si>
+    <t>Points close to a straight diagonal line. Heavy tails or an S-curve indicate non-normal errors. Check QQ Correlation (Cell P10): below 0.98 = mild concern, below 0.95 = stronger concern. The chart title itself shows the live r and appends a '— check normality' warning when it falls below 0.95, matching the table's red threshold.</t>
+  </si>
+  <si>
+    <t>Points close to a 45° line. A bow or fan shape confirms the same problems seen in Residuals vs. Fitted but from a different angle. The chart title shows the response name and the live Adjusted R², so the fit's headline quality is on the plot itself.</t>
+  </si>
+  <si>
+    <t>Spikes above F.INV(0.5, p, n-p) — the median of the reference F distribution, so the bar to beat scales with the model's own size — mark observations with outsized influence on the fitted coefficients. Bars are ordered by observation number. The title prints the live cutoff, so the bar to beat is visible on the plot itself, and bars above it carry data labels naming the row. Inspect those rows for data entry errors or genuine outliers before removing them. Remove outliers only when you have a definitive, non-statistical reason to believe the data point is invalid, comes from a different population, or disproportionately distorts the analysis. Never filter out data solely because it is an extreme statistical value, as doing so can introduce bias and erase genuine insights.</t>
+  </si>
+  <si>
+    <t>High leverage alone is not a problem. Combined high leverage and large residual (top-right or bottom-right of the plot) = influential outlier. Hat &gt; 2p/n is flagged red; Hat &gt; 3p/n is additionally bold. The title prints the live mean leverage (p/n), so 'Hat &gt; 2p/n' reads directly as 'more than twice the printed mean.'</t>
+  </si>
+  <si>
+    <t>PRESS residuals inflate the ordinary residual by leverage. Bars are ordered by observation number. Large values (|PRESS| &gt; 2 × SE yellow, &gt; 3 × SE red) flag observations whose removal would substantially shift the fitted model. The chart title carries the live PRESS total.</t>
+  </si>
+  <si>
+    <t>These thresholds surface in three places: the flagged cells named above, the diagnostic and audit cells the table cites, and the chart titles and data labels on the Regression sheet — a chart can be judged against its own printed cutoff without scrolling back to its source cell.</t>
   </si>
 </sst>
 </file>
@@ -916,17 +995,17 @@
     </row>
     <row r="6" spans="1:1" ht="105" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
     </row>
     <row r="9" spans="1:1" ht="180" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
     </row>
     <row r="10" spans="1:1" ht="90" x14ac:dyDescent="0.25">
@@ -934,9 +1013,9 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:1" ht="360" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:1" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>105</v>
+        <v>133</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
@@ -966,17 +1045,17 @@
     </row>
     <row r="20" spans="1:1" ht="120" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>95</v>
+        <v>134</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
     </row>
     <row r="23" spans="1:1" ht="120" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>106</v>
+        <v>99</v>
       </c>
     </row>
   </sheetData>
@@ -986,7 +1065,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1687EF57-B6EB-444E-A46B-98E7D5CA1EC6}">
-  <dimension ref="A1:D37"/>
+  <dimension ref="A1:D38"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.7109375" customWidth="1"/>
@@ -1002,14 +1081,14 @@
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
     </row>
-    <row r="2" spans="1:4" ht="90" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" ht="225" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>11</v>
+        <v>159</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B4" s="5"/>
       <c r="C4" s="5"/>
@@ -1017,63 +1096,63 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="C5" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="D5" s="4" t="s">
         <v>15</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C6" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="D6" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D6" s="2" t="s">
+    </row>
+    <row r="7" spans="1:4" ht="105" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" ht="60" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
+      <c r="B7" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="C7" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="D7" s="2" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="75" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="B8" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>26</v>
-      </c>
       <c r="D8" s="2" t="s">
-        <v>27</v>
+        <v>161</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
@@ -1081,77 +1160,77 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="C11" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="D11" s="4" t="s">
         <v>15</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="240" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B12" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C12" s="2" t="s">
+      <c r="B13" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="C13" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="105" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" ht="195" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
+      <c r="B14" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="C14" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="C13" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="60" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
+      <c r="D14" s="2" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="90" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B15" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C14" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="75" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>39</v>
-      </c>
       <c r="D15" s="2" t="s">
-        <v>40</v>
+        <v>164</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="B17" s="5"/>
       <c r="C17" s="5"/>
@@ -1159,243 +1238,248 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="B31" s="5"/>
-      <c r="C31" s="5"/>
+        <v>69</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="150" x14ac:dyDescent="0.25">
+      <c r="A30" s="2" t="s">
+        <v>165</v>
+      </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="B32" s="5"/>
+      <c r="C32" s="5"/>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" ht="120" x14ac:dyDescent="0.25">
+      <c r="A34" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C34" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="B32" s="4" t="s">
+    </row>
+    <row r="35" spans="1:3" ht="105" x14ac:dyDescent="0.25">
+      <c r="A35" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="C32" s="4" t="s">
+      <c r="B35" s="2" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="33" spans="1:3" ht="120" x14ac:dyDescent="0.25">
-      <c r="A33" s="2" t="s">
+      <c r="C35" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="B33" s="2" t="s">
+    </row>
+    <row r="36" spans="1:3" ht="120" x14ac:dyDescent="0.25">
+      <c r="A36" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="C33" s="2" t="s">
+      <c r="B36" s="2" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="34" spans="1:3" ht="105" x14ac:dyDescent="0.25">
-      <c r="A34" s="2" t="s">
+      <c r="C36" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="B34" s="2" t="s">
+    </row>
+    <row r="37" spans="1:3" ht="240" x14ac:dyDescent="0.25">
+      <c r="A37" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C34" s="2" t="s">
+      <c r="B37" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="C37" s="2" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="35" spans="1:3" ht="120" x14ac:dyDescent="0.25">
-      <c r="A35" s="2" t="s">
+    <row r="38" spans="1:3" ht="150" x14ac:dyDescent="0.25">
+      <c r="A38" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="B35" s="2" t="s">
+      <c r="B38" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="C35" s="2" t="s">
+      <c r="C38" s="2" t="s">
         <v>87</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" ht="240" x14ac:dyDescent="0.25">
-      <c r="A36" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="B36" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" ht="150" x14ac:dyDescent="0.25">
-      <c r="A37" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="B37" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="C37" s="2" t="s">
-        <v>92</v>
       </c>
     </row>
   </sheetData>
@@ -1405,7 +1489,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D1D5C19-8245-4AA6-BFBC-8BFCB51F135C}">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.7109375" customWidth="1"/>
@@ -1416,7 +1500,7 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -1424,119 +1508,216 @@
     </row>
     <row r="2" spans="1:4" ht="255" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>110</v>
+        <v>135</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>112</v>
+        <v>136</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="150" x14ac:dyDescent="0.25">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="165" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>115</v>
+        <v>129</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>116</v>
+        <v>130</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>117</v>
+        <v>131</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>118</v>
+        <v>132</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="165" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="225" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="D7" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="180" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="C7" s="2" t="s">
+    </row>
+    <row r="8" spans="1:4" ht="180" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="B8" s="2" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" ht="225" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
+      <c r="C8" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="D8" s="2" t="s">
         <v>128</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="255" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>131</v>
+        <v>121</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>132</v>
+        <v>122</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>133</v>
+        <v>123</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="180" x14ac:dyDescent="0.25">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="150" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>135</v>
+        <v>105</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="180" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="B13" s="3"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+    </row>
+    <row r="14" spans="1:4" ht="165" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="B16" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="C10" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="165" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
+      <c r="C16" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="105" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B17" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C17" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="D17" s="2" t="s">
         <v>142</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="105" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="90" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="90" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="90" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>158</v>
       </c>
     </row>
   </sheetData>

</xml_diff>